<commit_message>
Adds new calcs for linearity measurements. Tests with new system holding the servo motor.
</commit_message>
<xml_diff>
--- a/RMTest-.xlsx
+++ b/RMTest-.xlsx
@@ -14,12 +14,69 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Soll-Winkel [°]</t>
+  </si>
+  <si>
+    <t>Soll-Spannung [V]</t>
+  </si>
+  <si>
+    <t>Ist-Spannung [V]</t>
+  </si>
+  <si>
+    <t>Ist-Winkel [°]</t>
+  </si>
+  <si>
+    <t>Realer Winkel zur Mitte [°]</t>
+  </si>
   <si>
     <t>Soll-Spannung Real [V]</t>
   </si>
   <si>
     <t>Linearität</t>
+  </si>
+  <si>
+    <t>Mittelposition</t>
+  </si>
+  <si>
+    <t>Start aktiver Bereich CW (Drehrichtung-)</t>
+  </si>
+  <si>
+    <t>50° CW (25% aktiver Bereich)(Drehrichtung-)</t>
+  </si>
+  <si>
+    <t>75° CW (50% aktiver Bereich)(Drehrichtung-)</t>
+  </si>
+  <si>
+    <t>100° CW (75% aktiver Bereich)(Drehrichtung-)</t>
+  </si>
+  <si>
+    <t>Ende aktiver Bereich CW (Drehrichtung-)(11) 10V</t>
+  </si>
+  <si>
+    <t>Mechanisches Ende CW (Drehrichtung-)</t>
+  </si>
+  <si>
+    <t>Start aktiver Bereich CCW (Drehrichtung+)</t>
+  </si>
+  <si>
+    <t>50° CCW (25% aktiver Bereich)(Drehrichtung+)</t>
+  </si>
+  <si>
+    <t>75° CCW (50% aktiver Bereich)(Drehrichtung+)</t>
+  </si>
+  <si>
+    <t>100° CCW (75% aktiver Bereich)(Drehrichtung+)</t>
+  </si>
+  <si>
+    <t>Ende aktiver Bereich CCW (Drehrichtung+)(13) 0V</t>
+  </si>
+  <si>
+    <t>Mechanisches Ende CCW (Drehrichtung+)</t>
   </si>
   <si>
     <t>Totzone</t>
@@ -67,12 +124,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF86A5A"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -87,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -103,6 +166,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -398,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="44.7109375" customWidth="1"/>
@@ -410,38 +476,388 @@
     <col min="8" max="8" width="20.7109375" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="5" customFormat="1" ht="35" customHeight="1">
+    <row r="1" spans="1:8" s="5" customFormat="1" ht="35" customHeight="1">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="C1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="1">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2">
+        <v>5</v>
+      </c>
+      <c r="D2" s="3">
+        <v>4.957</v>
+      </c>
+      <c r="E2" s="1">
+        <v>-0</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0</v>
+      </c>
+      <c r="G2" s="3">
+        <v>5.016</v>
+      </c>
+      <c r="H2" s="4">
+        <v>-0.005848</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
+        <v>9</v>
+      </c>
+      <c r="B3" s="1">
+        <v>25</v>
+      </c>
+      <c r="C3" s="2">
+        <v>5</v>
+      </c>
+      <c r="D3" s="3">
+        <v>4.961</v>
+      </c>
+      <c r="E3" s="1">
+        <v>26.1</v>
+      </c>
+      <c r="F3" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
+        <v>10</v>
+      </c>
+      <c r="B4" s="1">
+        <v>50</v>
+      </c>
+      <c r="C4" s="2">
+        <v>6.25</v>
+      </c>
+      <c r="D4" s="3">
+        <v>6.169</v>
+      </c>
+      <c r="E4" s="1">
+        <v>49.8</v>
+      </c>
+      <c r="F4" s="1">
+        <v>23.7</v>
+      </c>
+      <c r="G4" s="3">
+        <v>6.214</v>
+      </c>
+      <c r="H4" s="4">
+        <v>-0.004505</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+        <v>11</v>
+      </c>
+      <c r="B5" s="1">
+        <v>75</v>
+      </c>
+      <c r="C5" s="2">
+        <v>7.5</v>
+      </c>
+      <c r="D5" s="3">
+        <v>7.449</v>
+      </c>
+      <c r="E5" s="1">
+        <v>74.8</v>
+      </c>
+      <c r="F5" s="1">
+        <v>48.7</v>
+      </c>
+      <c r="G5" s="3">
+        <v>7.474</v>
+      </c>
+      <c r="H5" s="4">
+        <v>-0.002512</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="1">
+        <v>100</v>
+      </c>
+      <c r="C6" s="2">
+        <v>8.75</v>
+      </c>
+      <c r="D6" s="3">
+        <v>8.731</v>
+      </c>
+      <c r="E6" s="1">
+        <v>99.7</v>
+      </c>
+      <c r="F6" s="1">
+        <v>73.7</v>
+      </c>
+      <c r="G6" s="3">
+        <v>8.734999999999999</v>
+      </c>
+      <c r="H6" s="4">
+        <v>-0.000374</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="1">
+        <v>125</v>
+      </c>
+      <c r="C7" s="2">
+        <v>10</v>
+      </c>
+      <c r="D7" s="3">
+        <v>9.999000000000001</v>
+      </c>
+      <c r="E7" s="1">
+        <v>124.8</v>
+      </c>
+      <c r="F7" s="1">
+        <v>98.7</v>
+      </c>
+      <c r="G7" s="3">
+        <v>10</v>
+      </c>
+      <c r="H7" s="4">
+        <v>-9.6E-05</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="1">
+        <v>165.9</v>
+      </c>
+      <c r="C8" s="2">
+        <v>10</v>
+      </c>
+      <c r="D8" s="3">
+        <v>9.999000000000001</v>
+      </c>
+      <c r="E8" s="1">
+        <v>165.9</v>
+      </c>
+      <c r="F8" s="1">
+        <v>139.8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="1">
+        <v>-25</v>
+      </c>
+      <c r="C9" s="2">
         <v>5</v>
+      </c>
+      <c r="D9" s="3">
+        <v>4.957</v>
+      </c>
+      <c r="E9" s="1">
+        <v>-24.6</v>
+      </c>
+      <c r="F9" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="1">
+        <v>-50</v>
+      </c>
+      <c r="C10" s="2">
+        <v>3.75</v>
+      </c>
+      <c r="D10" s="3">
+        <v>3.675</v>
+      </c>
+      <c r="E10" s="1">
+        <v>-50.1</v>
+      </c>
+      <c r="F10" s="1">
+        <v>-25.6</v>
+      </c>
+      <c r="G10" s="3">
+        <v>3.724</v>
+      </c>
+      <c r="H10" s="4">
+        <v>-0.004868</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="1">
+        <v>-75</v>
+      </c>
+      <c r="C11" s="2">
+        <v>2.5</v>
+      </c>
+      <c r="D11" s="3">
+        <v>2.434</v>
+      </c>
+      <c r="E11" s="1">
+        <v>-75.09999999999999</v>
+      </c>
+      <c r="F11" s="1">
+        <v>-50.5</v>
+      </c>
+      <c r="G11" s="3">
+        <v>2.463</v>
+      </c>
+      <c r="H11" s="4">
+        <v>-0.002901</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="1">
+        <v>-100</v>
+      </c>
+      <c r="C12" s="2">
+        <v>1.25</v>
+      </c>
+      <c r="D12" s="3">
+        <v>1.187</v>
+      </c>
+      <c r="E12" s="1">
+        <v>-100.1</v>
+      </c>
+      <c r="F12" s="1">
+        <v>-75.5</v>
+      </c>
+      <c r="G12" s="3">
+        <v>1.203</v>
+      </c>
+      <c r="H12" s="4">
+        <v>-0.001536</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="1">
+        <v>-125</v>
+      </c>
+      <c r="C13" s="2">
+        <v>0</v>
+      </c>
+      <c r="D13" s="3">
+        <v>0.001</v>
+      </c>
+      <c r="E13" s="1">
+        <v>-123.9</v>
+      </c>
+      <c r="F13" s="1">
+        <v>-99.3</v>
+      </c>
+      <c r="G13" s="3">
+        <v>-0</v>
+      </c>
+      <c r="H13" s="4">
+        <v>0.000139</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="1">
+        <v>-165.9</v>
+      </c>
+      <c r="C14" s="2">
+        <v>0</v>
+      </c>
+      <c r="D14" s="3">
+        <v>0</v>
+      </c>
+      <c r="E14" s="1">
+        <v>-165.9</v>
+      </c>
+      <c r="F14" s="1">
+        <v>-141.3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="1">
+        <v>50.6</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H16" s="6">
+        <v>0.000139</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="1">
+        <v>98.7</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H17" s="6">
+        <v>-0.005848</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="1">
+        <v>99.3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" t="s">
+        <v>24</v>
+      </c>
+      <c r="B20" s="1">
+        <v>198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adds tolerances for individual potentiometer models. Modified timeouts and debugs for goal reaching. Fine-tuned break out currents for smoother measurementes. Adds Excel marking for linearity errors. Changes outputs to stop overwriting files.
</commit_message>
<xml_diff>
--- a/RMTest-.xlsx
+++ b/RMTest-.xlsx
@@ -516,16 +516,16 @@
         <v>4.957</v>
       </c>
       <c r="E2" s="1">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="F2" s="1">
         <v>0</v>
       </c>
       <c r="G2" s="3">
-        <v>5.016</v>
+        <v>5.035</v>
       </c>
       <c r="H2" s="4">
-        <v>-0.005848</v>
+        <v>-0.007791</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -539,10 +539,10 @@
         <v>5</v>
       </c>
       <c r="D3" s="3">
-        <v>4.961</v>
+        <v>4.957</v>
       </c>
       <c r="E3" s="1">
-        <v>26.1</v>
+        <v>26.6</v>
       </c>
       <c r="F3" s="1">
         <v>0</v>
@@ -559,19 +559,19 @@
         <v>6.25</v>
       </c>
       <c r="D4" s="3">
-        <v>6.169</v>
+        <v>6.135</v>
       </c>
       <c r="E4" s="1">
         <v>49.8</v>
       </c>
       <c r="F4" s="1">
-        <v>23.7</v>
+        <v>23.2</v>
       </c>
       <c r="G4" s="3">
-        <v>6.214</v>
+        <v>6.206</v>
       </c>
       <c r="H4" s="4">
-        <v>-0.004505</v>
+        <v>-0.007144</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -585,19 +585,19 @@
         <v>7.5</v>
       </c>
       <c r="D5" s="3">
-        <v>7.449</v>
+        <v>7.425</v>
       </c>
       <c r="E5" s="1">
         <v>74.8</v>
       </c>
       <c r="F5" s="1">
-        <v>48.7</v>
+        <v>48.2</v>
       </c>
       <c r="G5" s="3">
-        <v>7.474</v>
+        <v>7.466</v>
       </c>
       <c r="H5" s="4">
-        <v>-0.002512</v>
+        <v>-0.004144</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -611,19 +611,19 @@
         <v>8.75</v>
       </c>
       <c r="D6" s="3">
-        <v>8.731</v>
+        <v>8.721</v>
       </c>
       <c r="E6" s="1">
         <v>99.7</v>
       </c>
       <c r="F6" s="1">
-        <v>73.7</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="G6" s="3">
-        <v>8.734999999999999</v>
+        <v>8.726000000000001</v>
       </c>
       <c r="H6" s="4">
-        <v>-0.000374</v>
+        <v>-0.00052</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -640,16 +640,16 @@
         <v>9.999000000000001</v>
       </c>
       <c r="E7" s="1">
-        <v>124.8</v>
+        <v>124.9</v>
       </c>
       <c r="F7" s="1">
-        <v>98.7</v>
+        <v>98.3</v>
       </c>
       <c r="G7" s="3">
-        <v>10</v>
+        <v>9.999000000000001</v>
       </c>
       <c r="H7" s="4">
-        <v>-9.6E-05</v>
+        <v>2E-06</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -657,7 +657,7 @@
         <v>14</v>
       </c>
       <c r="B8" s="1">
-        <v>165.9</v>
+        <v>165.5</v>
       </c>
       <c r="C8" s="2">
         <v>10</v>
@@ -666,10 +666,10 @@
         <v>9.999000000000001</v>
       </c>
       <c r="E8" s="1">
-        <v>165.9</v>
+        <v>165.5</v>
       </c>
       <c r="F8" s="1">
-        <v>139.8</v>
+        <v>138.9</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -683,10 +683,10 @@
         <v>5</v>
       </c>
       <c r="D9" s="3">
-        <v>4.957</v>
+        <v>4.948</v>
       </c>
       <c r="E9" s="1">
-        <v>-24.6</v>
+        <v>-24</v>
       </c>
       <c r="F9" s="1">
         <v>0</v>
@@ -703,19 +703,19 @@
         <v>3.75</v>
       </c>
       <c r="D10" s="3">
-        <v>3.675</v>
+        <v>3.652</v>
       </c>
       <c r="E10" s="1">
-        <v>-50.1</v>
+        <v>-50.2</v>
       </c>
       <c r="F10" s="1">
-        <v>-25.6</v>
+        <v>-26.3</v>
       </c>
       <c r="G10" s="3">
-        <v>3.724</v>
+        <v>3.709</v>
       </c>
       <c r="H10" s="4">
-        <v>-0.004868</v>
+        <v>-0.005662</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -729,19 +729,19 @@
         <v>2.5</v>
       </c>
       <c r="D11" s="3">
-        <v>2.434</v>
+        <v>2.416</v>
       </c>
       <c r="E11" s="1">
-        <v>-75.09999999999999</v>
+        <v>-75.2</v>
       </c>
       <c r="F11" s="1">
-        <v>-50.5</v>
+        <v>-51.2</v>
       </c>
       <c r="G11" s="3">
-        <v>2.463</v>
+        <v>2.449</v>
       </c>
       <c r="H11" s="4">
-        <v>-0.002901</v>
+        <v>-0.003307</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -755,19 +755,19 @@
         <v>1.25</v>
       </c>
       <c r="D12" s="3">
-        <v>1.187</v>
+        <v>1.177</v>
       </c>
       <c r="E12" s="1">
         <v>-100.1</v>
       </c>
       <c r="F12" s="1">
-        <v>-75.5</v>
+        <v>-76.09999999999999</v>
       </c>
       <c r="G12" s="3">
-        <v>1.203</v>
+        <v>1.193</v>
       </c>
       <c r="H12" s="4">
-        <v>-0.001536</v>
+        <v>-0.001627</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -781,19 +781,19 @@
         <v>0</v>
       </c>
       <c r="D13" s="3">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="E13" s="1">
-        <v>-123.9</v>
+        <v>-123.7</v>
       </c>
       <c r="F13" s="1">
-        <v>-99.3</v>
+        <v>-99.8</v>
       </c>
       <c r="G13" s="3">
         <v>-0</v>
       </c>
       <c r="H13" s="4">
-        <v>0.000139</v>
+        <v>2E-05</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -801,7 +801,7 @@
         <v>20</v>
       </c>
       <c r="B14" s="1">
-        <v>-165.9</v>
+        <v>-165.5</v>
       </c>
       <c r="C14" s="2">
         <v>0</v>
@@ -810,10 +810,10 @@
         <v>0</v>
       </c>
       <c r="E14" s="1">
-        <v>-165.9</v>
+        <v>-165.5</v>
       </c>
       <c r="F14" s="1">
-        <v>-141.3</v>
+        <v>-141.5</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -821,13 +821,13 @@
         <v>21</v>
       </c>
       <c r="B16" s="1">
-        <v>50.6</v>
+        <v>50.5</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="H16" s="6">
-        <v>0.000139</v>
+      <c r="H16" s="4">
+        <v>2E-05</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -835,13 +835,13 @@
         <v>22</v>
       </c>
       <c r="B17" s="1">
-        <v>98.7</v>
+        <v>98.3</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>26</v>
       </c>
       <c r="H17" s="6">
-        <v>-0.005848</v>
+        <v>-0.007791</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -849,7 +849,7 @@
         <v>23</v>
       </c>
       <c r="B18" s="1">
-        <v>99.3</v>
+        <v>99.8</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -857,7 +857,7 @@
         <v>24</v>
       </c>
       <c r="B20" s="1">
-        <v>198</v>
+        <v>198.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>